<commit_message>
Published state of ETDataset for deploy 2026-02
</commit_message>
<xml_diff>
--- a/analyses/7_services_analysis.xlsx
+++ b/analyses/7_services_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10110"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathijsbijkerk/Github/etdataset/analyses/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyradehaan/github/etdataset/analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BA178EE-A6B7-FD43-A491-70E9C079A6B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CBBE78-021D-8640-97BC-7C1E47A0EE28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13360" yWindow="-28300" windowWidth="25600" windowHeight="27360" tabRatio="929" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" tabRatio="929" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Sheet" sheetId="34" r:id="rId1"/>
@@ -39,12 +39,10 @@
     <sheet name="csv_ps_final_demand_electricity" sheetId="55" r:id="rId24"/>
     <sheet name="csv_ps_final_demand_wood_p" sheetId="58" r:id="rId25"/>
     <sheet name="csv_cooling_useful_insulation" sheetId="63" r:id="rId26"/>
-    <sheet name="csv_light_saving_detection" sheetId="66" r:id="rId27"/>
-    <sheet name="csv_light_saving_control" sheetId="67" r:id="rId28"/>
-    <sheet name="csv_ps_sector_electricity" sheetId="68" r:id="rId29"/>
+    <sheet name="csv_ps_sector_electricity" sheetId="68" r:id="rId27"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId30"/>
+    <externalReference r:id="rId28"/>
   </externalReferences>
   <definedNames>
     <definedName name="base_year">Dashboard!$E$12</definedName>
@@ -166,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="621">
   <si>
     <t>Changelog</t>
   </si>
@@ -1492,24 +1490,6 @@
     <t>buildings_useful_demand_after_insulation_cooling</t>
   </si>
   <si>
-    <t>buildings_useful_demand_light_child_share</t>
-  </si>
-  <si>
-    <t>buildings_useful_demand_after_motion_detection_light</t>
-  </si>
-  <si>
-    <t>buildings_lighting_savings_from_motion_detection_light</t>
-  </si>
-  <si>
-    <t>buildings_useful_demand_after_motion_detection_light_child_share</t>
-  </si>
-  <si>
-    <t>buildings_useful_demand_after_motion_detection_daylight_control_light</t>
-  </si>
-  <si>
-    <t>buildings_lighting_savings_from_daylight_control_light</t>
-  </si>
-  <si>
     <t>Added shares that define converters related to "savings" (RD)</t>
   </si>
   <si>
@@ -1769,12 +1749,6 @@
   </si>
   <si>
     <t>The ETM graph contains a number of converters that are used to model future energy saving effects of improved insulation. The inluence of these converters is set to 'zero' in the 'present' scenario:</t>
-  </si>
-  <si>
-    <t>Current savings in useful demand of lighting accomplished by motion detection</t>
-  </si>
-  <si>
-    <t>Current savings in useful demand of lighting accomplished by daylight control</t>
   </si>
   <si>
     <t>Removing converters
@@ -1836,12 +1810,6 @@
     <t>services_biomass_used_in appliances</t>
   </si>
   <si>
-    <t>services_savings_lighting_motion_detection</t>
-  </si>
-  <si>
-    <t>services_savings_lighting_daylight_control</t>
-  </si>
-  <si>
     <t>services_space_heating_share_electric_heat_pump_with_storage</t>
   </si>
   <si>
@@ -2164,9 +2132,6 @@
     <t>buildings_space_heater_district_heating_ht_steam_hot_water</t>
   </si>
   <si>
-    <t>Mathijs Bijkerk</t>
-  </si>
-  <si>
     <t>Quintel</t>
   </si>
   <si>
@@ -2195,6 +2160,12 @@
   </si>
   <si>
     <t>Add surface water technologies to export CSVs with zero share.</t>
+  </si>
+  <si>
+    <t>Remove intelligent light control keys</t>
+  </si>
+  <si>
+    <t>Kyra de Haan</t>
   </si>
 </sst>
 </file>
@@ -9751,7 +9722,7 @@
       </c>
       <c r="C5" s="24">
         <f>MAX(Changelog!D:D)</f>
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
       <c r="D5" s="7"/>
     </row>
@@ -9779,8 +9750,8 @@
       <c r="B8" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="195" t="s">
-        <v>628</v>
+      <c r="C8" s="195">
+        <v>46041</v>
       </c>
       <c r="D8" s="7"/>
     </row>
@@ -9789,7 +9760,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D9" s="7"/>
     </row>
@@ -9798,7 +9769,7 @@
         <v>20</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>620</v>
+        <v>609</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -10002,7 +9973,7 @@
     </row>
     <row r="5" spans="2:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="372" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
       <c r="C5" s="374"/>
       <c r="D5" s="374"/>
@@ -10011,13 +9982,13 @@
     <row r="6" spans="2:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B7" s="190" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="C7" s="265" t="s">
         <v>336</v>
       </c>
       <c r="D7" s="157" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="E7" s="158" t="s">
         <v>341</v>
@@ -10067,7 +10038,7 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B12" s="261" t="s">
-        <v>578</v>
+        <v>568</v>
       </c>
       <c r="C12" s="159"/>
       <c r="D12" s="212"/>
@@ -10238,7 +10209,7 @@
     <row r="27" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B27" s="262"/>
       <c r="C27" s="16" t="s">
-        <v>597</v>
+        <v>587</v>
       </c>
       <c r="D27" s="211" t="e">
         <f>SUM(D22:D25)</f>
@@ -10252,7 +10223,7 @@
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" s="262"/>
       <c r="C28" s="16" t="s">
-        <v>595</v>
+        <v>585</v>
       </c>
       <c r="D28" s="211">
         <f>SUM('Final demand per energy carrier'!J39)</f>
@@ -10327,10 +10298,10 @@
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:6" ht="48" x14ac:dyDescent="0.2">
       <c r="B7" s="190" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="C7" s="257" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="D7" s="265" t="s">
         <v>225</v>
@@ -10339,7 +10310,7 @@
         <v>345</v>
       </c>
       <c r="F7" s="158" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.2">
@@ -10354,7 +10325,7 @@
     <row r="9" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B9" s="262"/>
       <c r="C9" s="58" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>121</v>
@@ -10425,7 +10396,7 @@
       <c r="B14" s="262"/>
       <c r="C14" s="58"/>
       <c r="D14" s="16" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="E14" s="177" t="e">
         <f>'Technology split final demand'!G17</f>
@@ -10488,7 +10459,7 @@
       <c r="B19" s="262"/>
       <c r="C19" s="58"/>
       <c r="D19" s="16" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="E19" s="177" t="e">
         <f>'Technology split final demand'!G27</f>
@@ -10613,7 +10584,7 @@
     </row>
     <row r="5" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="372" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="C5" s="374"/>
       <c r="D5" s="374"/>
@@ -10649,28 +10620,28 @@
         <v>130</v>
       </c>
       <c r="D9" s="99" t="s">
-        <v>568</v>
+        <v>558</v>
       </c>
       <c r="E9" s="65" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="F9" s="65" t="s">
-        <v>579</v>
+        <v>569</v>
       </c>
       <c r="G9" s="65" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="H9" s="65" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="I9" s="65" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="J9" s="65" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
@@ -11138,7 +11109,7 @@
     <row r="36" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B36" s="28"/>
       <c r="C36" t="s">
-        <v>569</v>
+        <v>559</v>
       </c>
       <c r="D36" s="71"/>
       <c r="E36" s="242" t="e">
@@ -11184,7 +11155,7 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B38" s="362" t="s">
-        <v>595</v>
+        <v>585</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="5"/>
@@ -11199,30 +11170,30 @@
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B39" s="28"/>
       <c r="C39" s="1" t="s">
-        <v>596</v>
+        <v>586</v>
       </c>
       <c r="D39" s="7"/>
       <c r="E39" s="369" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="F39" s="369" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G39" s="369" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H39" s="369" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I39" s="369" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J39" s="242" t="str">
         <f>Dashboard!E29</f>
         <v/>
       </c>
       <c r="K39" s="370" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
@@ -11239,7 +11210,7 @@
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B41" s="362" t="s">
-        <v>572</v>
+        <v>562</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
@@ -11271,7 +11242,7 @@
     <row r="43" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B43" s="28"/>
       <c r="C43" t="s">
-        <v>570</v>
+        <v>560</v>
       </c>
       <c r="D43" s="71"/>
       <c r="E43" s="242" t="e">
@@ -11287,16 +11258,16 @@
         <v>#DIV/0!</v>
       </c>
       <c r="H43" s="350" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I43" s="350" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J43" s="350" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="K43" s="358" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
     </row>
     <row r="44" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -11378,7 +11349,7 @@
     <row r="6" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B7" s="25" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="C7" s="51"/>
       <c r="D7" s="26"/>
@@ -11574,7 +11545,7 @@
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B17" s="35"/>
       <c r="C17" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="D17" s="175">
         <f>Dashboard!E50</f>
@@ -11741,7 +11712,7 @@
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B27" s="262"/>
       <c r="C27" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="D27" s="279">
         <f>Dashboard!E57</f>
@@ -12119,7 +12090,7 @@
         <v>270</v>
       </c>
       <c r="D9" s="65" t="s">
-        <v>580</v>
+        <v>570</v>
       </c>
       <c r="E9" s="65" t="s">
         <v>271</v>
@@ -12140,10 +12111,10 @@
         <v>285</v>
       </c>
       <c r="K9" s="250" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="L9" s="136" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.2">
@@ -12223,13 +12194,13 @@
     </row>
     <row r="17" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J17" s="244" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="K17" s="192"/>
     </row>
     <row r="18" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J18" s="245" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="K18" s="246"/>
     </row>
@@ -12249,13 +12220,13 @@
     </row>
     <row r="21" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J21" s="245" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="K21" s="246"/>
     </row>
     <row r="22" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J22" s="245" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="K22" s="246"/>
     </row>
@@ -12265,7 +12236,7 @@
     </row>
     <row r="24" spans="10:11" x14ac:dyDescent="0.2">
       <c r="J24" s="247" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="K24" s="248">
         <f>K11-Final_demand_residences</f>
@@ -12370,10 +12341,10 @@
         <v>296</v>
       </c>
       <c r="E8" s="99" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="F8" s="99" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="G8" s="180" t="s">
         <v>297</v>
@@ -12521,7 +12492,7 @@
     <row r="15" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B15" s="33"/>
       <c r="C15" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
       <c r="D15" s="175" t="e">
         <f>'Technology split final demand'!G17</f>
@@ -12746,7 +12717,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="194" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
       <c r="B5" s="266" t="e">
         <f>'Technology shares'!F14</f>
@@ -12755,7 +12726,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="194" t="s">
-        <v>626</v>
+        <v>615</v>
       </c>
       <c r="B6" s="266">
         <v>0</v>
@@ -12820,7 +12791,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="228" t="s">
-        <v>612</v>
+        <v>602</v>
       </c>
       <c r="B5" s="266" t="e">
         <f>'Technology shares'!F19</f>
@@ -12829,7 +12800,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>627</v>
+        <v>616</v>
       </c>
       <c r="B6" s="266">
         <v>0</v>
@@ -12854,7 +12825,7 @@
   <sheetPr codeName="Sheet2">
     <tabColor theme="2"/>
   </sheetPr>
-  <dimension ref="B2:E53"/>
+  <dimension ref="B2:E54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -13094,7 +13065,7 @@
         <v>41485</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="D23" s="290">
         <v>1.18</v>
@@ -13106,7 +13077,7 @@
         <v>41485</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="D24" s="290">
         <v>1.18</v>
@@ -13118,7 +13089,7 @@
         <v>41486</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="D25" s="290">
         <v>1.19</v>
@@ -13130,7 +13101,7 @@
         <v>41487</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="D26" s="290">
         <v>1.19</v>
@@ -13142,7 +13113,7 @@
         <v>41499</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="D27" s="289">
         <v>1.2</v>
@@ -13154,7 +13125,7 @@
         <v>41500</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="D28" s="290">
         <v>1.21</v>
@@ -13166,7 +13137,7 @@
         <v>41500</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="D29" s="289">
         <v>1.22</v>
@@ -13178,7 +13149,7 @@
         <v>41502</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="D30" s="289">
         <v>1.23</v>
@@ -13190,7 +13161,7 @@
         <v>41505</v>
       </c>
       <c r="C31" s="37" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="D31" s="289">
         <v>1.24</v>
@@ -13202,7 +13173,7 @@
         <v>41506</v>
       </c>
       <c r="C32" s="37" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="D32" s="289">
         <v>1.25</v>
@@ -13214,7 +13185,7 @@
         <v>41507</v>
       </c>
       <c r="C33" s="37" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="D33" s="289">
         <v>1.26</v>
@@ -13226,7 +13197,7 @@
         <v>41509</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="D34" s="289">
         <v>1.27</v>
@@ -13238,7 +13209,7 @@
         <v>41509</v>
       </c>
       <c r="C35" s="37" t="s">
-        <v>514</v>
+        <v>504</v>
       </c>
       <c r="D35" s="289">
         <v>1.28</v>
@@ -13247,10 +13218,10 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" s="287" t="s">
-        <v>521</v>
+        <v>511</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>521</v>
+        <v>511</v>
       </c>
       <c r="D36" s="289">
         <v>1.29</v>
@@ -13262,7 +13233,7 @@
         <v>41534</v>
       </c>
       <c r="C37" s="37" t="s">
-        <v>546</v>
+        <v>536</v>
       </c>
       <c r="D37" s="289">
         <v>1.3</v>
@@ -13274,7 +13245,7 @@
         <v>41542</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
       <c r="D38" s="289">
         <v>1.31</v>
@@ -13286,7 +13257,7 @@
         <v>41562</v>
       </c>
       <c r="C39" s="339" t="s">
-        <v>548</v>
+        <v>538</v>
       </c>
       <c r="D39" s="289">
         <v>1.32</v>
@@ -13298,7 +13269,7 @@
         <v>41578</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>576</v>
+        <v>566</v>
       </c>
       <c r="D40" s="289">
         <v>1.33</v>
@@ -13310,7 +13281,7 @@
         <v>41578</v>
       </c>
       <c r="C41" s="37" t="s">
-        <v>577</v>
+        <v>567</v>
       </c>
       <c r="D41" s="289">
         <v>1.34</v>
@@ -13322,7 +13293,7 @@
         <v>41782</v>
       </c>
       <c r="C42" s="37" t="s">
-        <v>582</v>
+        <v>572</v>
       </c>
       <c r="D42" s="289">
         <v>1.35</v>
@@ -13334,7 +13305,7 @@
         <v>41782</v>
       </c>
       <c r="C43" s="37" t="s">
-        <v>583</v>
+        <v>573</v>
       </c>
       <c r="D43" s="289">
         <v>1.36</v>
@@ -13346,7 +13317,7 @@
         <v>42600</v>
       </c>
       <c r="C44" s="37" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
       <c r="D44" s="289">
         <v>1.37</v>
@@ -13358,7 +13329,7 @@
         <v>44607</v>
       </c>
       <c r="C45" s="37" t="s">
-        <v>617</v>
+        <v>607</v>
       </c>
       <c r="D45" s="289">
         <v>1.38</v>
@@ -13367,10 +13338,10 @@
     </row>
     <row r="46" spans="2:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B46" s="338" t="s">
-        <v>621</v>
+        <v>610</v>
       </c>
       <c r="C46" s="37" t="s">
-        <v>622</v>
+        <v>611</v>
       </c>
       <c r="D46" s="289">
         <v>1.39</v>
@@ -13379,10 +13350,10 @@
     </row>
     <row r="47" spans="2:5" ht="51" x14ac:dyDescent="0.2">
       <c r="B47" s="338" t="s">
-        <v>623</v>
+        <v>612</v>
       </c>
       <c r="C47" s="37" t="s">
-        <v>624</v>
+        <v>613</v>
       </c>
       <c r="D47" s="289">
         <v>1.4</v>
@@ -13391,25 +13362,32 @@
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B48" s="338" t="s">
-        <v>628</v>
+        <v>617</v>
       </c>
       <c r="C48" s="37" t="s">
-        <v>629</v>
+        <v>618</v>
       </c>
       <c r="D48" s="289">
         <v>1.41</v>
       </c>
       <c r="E48" s="128"/>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B49" s="288"/>
-      <c r="C49" s="43"/>
-      <c r="D49" s="291"/>
+    <row r="49" spans="2:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B49" s="338">
+        <v>46041</v>
+      </c>
+      <c r="C49" s="37" t="s">
+        <v>619</v>
+      </c>
+      <c r="D49" s="289">
+        <v>1.42</v>
+      </c>
       <c r="E49" s="128"/>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B50" s="128"/>
-      <c r="D50" s="128"/>
+      <c r="B50" s="288"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="291"/>
       <c r="E50" s="128"/>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.2">
@@ -13419,9 +13397,14 @@
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B52" s="128"/>
+      <c r="D52" s="128"/>
+      <c r="E52" s="128"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B53" s="128"/>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B54" s="128"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13447,7 +13430,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="194" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -13584,7 +13567,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="194" t="s">
-        <v>584</v>
+        <v>574</v>
       </c>
       <c r="B3" s="266" t="e">
         <f>'Application shares'!E13</f>
@@ -13593,7 +13576,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="194" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
       <c r="B4" s="266" t="e">
         <f>'Application shares'!E14</f>
@@ -13602,7 +13585,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="194" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="B5" s="266" t="e">
         <f>'Application shares'!E15</f>
@@ -13886,132 +13869,6 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
-  <sheetPr codeName="Sheet32">
-    <tabColor theme="7" tint="0.39997558519241921"/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="47.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>366</v>
-      </c>
-      <c r="B2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>399</v>
-      </c>
-      <c r="B3" s="266">
-        <f>1-B4</f>
-        <v>0.96099999999999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>400</v>
-      </c>
-      <c r="B4" s="266">
-        <f>Dashboard!E69</f>
-        <v>3.9E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B5" s="266"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="266"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B7" s="266"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
-  <sheetPr codeName="Sheet33">
-    <tabColor theme="7" tint="0.39997558519241921"/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="61.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>366</v>
-      </c>
-      <c r="B2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>402</v>
-      </c>
-      <c r="B3" s="266">
-        <f>1-B4</f>
-        <v>0.94699999999999995</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>403</v>
-      </c>
-      <c r="B4" s="266">
-        <f>Dashboard!E70</f>
-        <v>5.2999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B5" s="266"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="266"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B7" s="266"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.39997558519241921"/>
@@ -14024,7 +13881,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="194" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -14037,7 +13894,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="194" t="s">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="B3" s="266" t="e">
         <f>'Application shares'!E27</f>
@@ -14046,7 +13903,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="194" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="B4" s="266" t="e">
         <f>'Application shares'!E28</f>
@@ -14164,7 +14021,7 @@
     </row>
     <row r="13" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="167" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="C13" s="59" t="s">
         <v>316</v>
@@ -14180,7 +14037,7 @@
     </row>
     <row r="15" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="282" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="C15" s="59" t="s">
         <v>342</v>
@@ -14188,7 +14045,7 @@
     </row>
     <row r="16" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="282" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="C16" s="59" t="s">
         <v>340</v>
@@ -14204,7 +14061,7 @@
     </row>
     <row r="18" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="117" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="C18" s="59" t="s">
         <v>314</v>
@@ -14215,7 +14072,7 @@
         <v>312</v>
       </c>
       <c r="C19" s="59" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -14236,106 +14093,106 @@
     </row>
     <row r="22" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="168" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="C22" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="168" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="C23" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="168" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="C24" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="168" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="C25" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="168" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="C26" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="168" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="C27" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="168" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="C28" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="168" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="C29" s="241" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="168" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="C30" s="241" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="168" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C31" s="241" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="168" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="C32" s="241" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="168" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="C33" s="241" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="34" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="168" t="s">
-        <v>603</v>
+        <v>593</v>
       </c>
       <c r="C34" s="241" t="s">
-        <v>604</v>
+        <v>594</v>
       </c>
     </row>
     <row r="35" spans="2:3" ht="28" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -14379,7 +14236,7 @@
     </row>
     <row r="6" spans="2:2" ht="80" x14ac:dyDescent="0.2">
       <c r="B6" s="104" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
@@ -14395,32 +14252,32 @@
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" s="121" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" s="53" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" s="53" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" s="53" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" s="121" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" s="121" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.2">
@@ -14939,14 +14796,14 @@
     <row r="15" spans="2:4" ht="47" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="36"/>
       <c r="C15" s="89" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="D15" s="38"/>
     </row>
     <row r="16" spans="2:4" ht="47" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="36"/>
       <c r="C16" s="89" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="D16" s="38"/>
     </row>
@@ -14956,7 +14813,7 @@
         <v>395</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -14965,7 +14822,7 @@
         <v>394</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -15258,7 +15115,7 @@
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B58" s="30" t="s">
-        <v>513</v>
+        <v>503</v>
       </c>
       <c r="C58" s="132" t="s">
         <v>263</v>
@@ -15354,7 +15211,7 @@
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" s="35" t="s">
-        <v>578</v>
+        <v>568</v>
       </c>
       <c r="C74" s="40" t="s">
         <v>265</v>
@@ -15727,7 +15584,7 @@
   <sheetPr codeName="Sheet7">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="B2:S71"/>
+  <dimension ref="B2:S68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -15754,7 +15611,7 @@
         <v>28</v>
       </c>
       <c r="K2" s="196" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="5"/>
@@ -15829,7 +15686,7 @@
       </c>
       <c r="F9" s="31"/>
       <c r="G9" s="31" t="s">
-        <v>520</v>
+        <v>510</v>
       </c>
       <c r="H9" s="31"/>
       <c r="I9" s="31" t="s">
@@ -15846,10 +15703,10 @@
         <v>93</v>
       </c>
       <c r="O9" s="222" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="P9" s="223" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.2">
@@ -15865,7 +15722,7 @@
       <c r="I10" s="14"/>
       <c r="J10" s="15"/>
       <c r="K10" s="340" t="s">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="L10" s="341" t="b">
         <f>IF(COUNTIF(P:P,0)+COUNTIF(P:P,FALSE)=0,TRUE,FALSE)</f>
@@ -15882,11 +15739,11 @@
       </c>
       <c r="D11" s="58"/>
       <c r="E11" s="127" t="s">
-        <v>625</v>
+        <v>614</v>
       </c>
       <c r="F11" s="14"/>
       <c r="G11" s="218" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="H11" s="216"/>
       <c r="I11" s="14"/>
@@ -15900,7 +15757,7 @@
       </c>
       <c r="M11" s="63"/>
       <c r="O11" s="199" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="P11" s="221">
         <f>IF(L11=TRUE,1,0)</f>
@@ -15910,7 +15767,7 @@
     <row r="12" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B12" s="33"/>
       <c r="C12" s="58" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="D12" s="58"/>
       <c r="E12" s="127">
@@ -15918,7 +15775,7 @@
       </c>
       <c r="F12" s="14"/>
       <c r="G12" s="218" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="H12" s="216"/>
       <c r="I12" s="14"/>
@@ -15927,7 +15784,7 @@
       <c r="L12" s="145"/>
       <c r="M12" s="63"/>
       <c r="O12" s="199" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="P12" s="221"/>
     </row>
@@ -15958,7 +15815,7 @@
       <c r="I14" s="14"/>
       <c r="J14" s="15"/>
       <c r="K14" s="62" t="s">
-        <v>571</v>
+        <v>561</v>
       </c>
       <c r="L14" s="145"/>
       <c r="M14" s="63"/>
@@ -15976,7 +15833,7 @@
       <c r="I15" s="14"/>
       <c r="J15" s="15"/>
       <c r="K15" s="53" t="s">
-        <v>574</v>
+        <v>564</v>
       </c>
       <c r="L15" s="347" t="e">
         <f>IF('Final demand per energy carrier'!E43&lt;0,FALSE,TRUE)</f>
@@ -16003,7 +15860,7 @@
       <c r="I16" s="14"/>
       <c r="J16" s="15"/>
       <c r="K16" s="53" t="s">
-        <v>573</v>
+        <v>563</v>
       </c>
       <c r="L16" s="347" t="e">
         <f>IF('Final demand per energy carrier'!F43&lt;0,FALSE,TRUE)</f>
@@ -16030,7 +15887,7 @@
       <c r="I17" s="14"/>
       <c r="J17" s="15"/>
       <c r="K17" s="53" t="s">
-        <v>575</v>
+        <v>565</v>
       </c>
       <c r="L17" s="347" t="e">
         <f>IF('Final demand per energy carrier'!G43&lt;0,FALSE,TRUE)</f>
@@ -16073,7 +15930,7 @@
       <c r="I19" s="297"/>
       <c r="J19" s="299"/>
       <c r="K19" s="55" t="s">
-        <v>567</v>
+        <v>557</v>
       </c>
       <c r="L19" s="365" t="b">
         <f>IF('Fuel aggregation'!J11=0,TRUE,'Fuel aggregation'!J11)</f>
@@ -16103,10 +15960,10 @@
     <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" s="35"/>
       <c r="C21" s="1" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E21" s="202">
         <f>Final_demand_residences</f>
@@ -16116,7 +15973,7 @@
       <c r="G21" s="218"/>
       <c r="H21" s="218"/>
       <c r="I21" s="1" t="s">
-        <v>551</v>
+        <v>541</v>
       </c>
       <c r="K21" s="53"/>
       <c r="L21" s="343"/>
@@ -16142,12 +15999,12 @@
         <v>101</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E23" s="204"/>
       <c r="F23" s="218"/>
       <c r="G23" s="218" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="H23" s="218"/>
       <c r="I23" s="21"/>
@@ -16156,7 +16013,7 @@
       <c r="L23" s="343"/>
       <c r="M23" s="54"/>
       <c r="O23" s="199" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="P23" s="221"/>
     </row>
@@ -16166,12 +16023,12 @@
         <v>104</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E24" s="205"/>
       <c r="F24" s="218"/>
       <c r="G24" s="218" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="H24" s="218"/>
       <c r="I24" s="21"/>
@@ -16180,7 +16037,7 @@
       <c r="L24" s="343"/>
       <c r="M24" s="54"/>
       <c r="O24" s="199" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
       <c r="P24" s="221"/>
     </row>
@@ -16190,12 +16047,12 @@
         <v>102</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E25" s="205"/>
       <c r="F25" s="218"/>
       <c r="G25" s="218" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="H25" s="218"/>
       <c r="I25" s="21"/>
@@ -16204,7 +16061,7 @@
       <c r="L25" s="343"/>
       <c r="M25" s="54"/>
       <c r="O25" s="199" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="P25" s="221"/>
     </row>
@@ -16235,7 +16092,7 @@
     <row r="28" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B28" s="35"/>
       <c r="C28" s="1" t="s">
-        <v>592</v>
+        <v>582</v>
       </c>
       <c r="E28" s="205"/>
       <c r="F28" s="214"/>
@@ -16245,17 +16102,17 @@
       <c r="L28" s="343"/>
       <c r="M28" s="54"/>
       <c r="O28" s="199" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="P28" s="221"/>
     </row>
     <row r="29" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B29" s="35"/>
       <c r="C29" s="1" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E29" s="205" t="str">
         <f>IF(E28="no",0,"")</f>
@@ -16263,12 +16120,12 @@
       </c>
       <c r="F29" s="214"/>
       <c r="G29" s="218" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="H29" s="218"/>
       <c r="I29" s="21"/>
       <c r="K29" s="62" t="s">
-        <v>594</v>
+        <v>584</v>
       </c>
       <c r="L29" s="347" t="b">
         <f>IF(E29&gt;=0,TRUE,E29)</f>
@@ -16279,7 +16136,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O29" s="199" t="s">
-        <v>591</v>
+        <v>581</v>
       </c>
       <c r="P29" s="221">
         <f>IF(L29=TRUE,1,0)</f>
@@ -16301,10 +16158,10 @@
     <row r="31" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B31" s="35"/>
       <c r="C31" s="1" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E31" s="344" t="e">
         <f>'Final demand per energy carrier'!J42</f>
@@ -16314,7 +16171,7 @@
       <c r="G31" s="218"/>
       <c r="H31" s="218"/>
       <c r="K31" s="62" t="s">
-        <v>564</v>
+        <v>554</v>
       </c>
       <c r="L31" s="347" t="e">
         <f>IF(E31&gt;0,TRUE,E31)</f>
@@ -16333,10 +16190,10 @@
     <row r="32" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B32" s="35"/>
       <c r="C32" s="1" t="s">
-        <v>566</v>
+        <v>556</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="E32" s="345" t="e">
         <f>SUM('Final demand per energy carrier'!E43:G43)</f>
@@ -16346,7 +16203,7 @@
       <c r="G32" s="218"/>
       <c r="H32" s="218"/>
       <c r="K32" s="62" t="s">
-        <v>565</v>
+        <v>555</v>
       </c>
       <c r="L32" s="347" t="e">
         <f>IF(E32&gt;0,TRUE,E32)</f>
@@ -16403,7 +16260,7 @@
     <row r="35" spans="2:19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="35"/>
       <c r="C35" s="1" t="s">
-        <v>516</v>
+        <v>506</v>
       </c>
       <c r="E35" s="344">
         <f>Final_demand_space_heating</f>
@@ -16427,14 +16284,14 @@
     <row r="37" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B37" s="35"/>
       <c r="C37" s="346" t="s">
-        <v>517</v>
+        <v>507</v>
       </c>
       <c r="E37" s="344">
         <f>'Final demand extracted from EB'!D13</f>
         <v>0</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>560</v>
+        <v>550</v>
       </c>
       <c r="K37" s="53"/>
       <c r="L37" s="146"/>
@@ -16445,14 +16302,14 @@
     <row r="38" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B38" s="35"/>
       <c r="C38" s="346" t="s">
-        <v>518</v>
+        <v>508</v>
       </c>
       <c r="E38" s="344">
         <f>'Final demand extracted from EB'!D9</f>
         <v>0</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>560</v>
+        <v>550</v>
       </c>
       <c r="K38" s="53"/>
       <c r="L38" s="146"/>
@@ -16463,14 +16320,14 @@
     <row r="39" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B39" s="35"/>
       <c r="C39" s="346" t="s">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="E39" s="344">
         <f>'Final demand extracted from EB'!D17</f>
         <v>0</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>560</v>
+        <v>550</v>
       </c>
       <c r="K39" s="53"/>
       <c r="L39" s="146"/>
@@ -16490,7 +16347,7 @@
     <row r="41" spans="2:19" ht="34" x14ac:dyDescent="0.2">
       <c r="B41" s="35"/>
       <c r="C41" s="90" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
       <c r="E41" s="344">
         <f>E35-SUM(E37:E39)</f>
@@ -16515,7 +16372,7 @@
     <row r="43" spans="2:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B43" s="35"/>
       <c r="C43" s="1" t="s">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="E43" s="57"/>
       <c r="K43" s="53"/>
@@ -16527,7 +16384,7 @@
     <row r="44" spans="2:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B44" s="35"/>
       <c r="C44" s="346" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
       <c r="E44" s="161"/>
       <c r="I44" s="21"/>
@@ -16535,14 +16392,14 @@
       <c r="L44" s="146"/>
       <c r="M44" s="294"/>
       <c r="O44" s="199" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="P44" s="221"/>
     </row>
     <row r="45" spans="2:19" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B45" s="35"/>
       <c r="C45" s="346" t="s">
-        <v>555</v>
+        <v>545</v>
       </c>
       <c r="E45" s="161"/>
       <c r="I45" s="21"/>
@@ -16550,7 +16407,7 @@
       <c r="L45" s="146"/>
       <c r="M45" s="294"/>
       <c r="O45" s="199" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="P45" s="221"/>
       <c r="S45" s="292"/>
@@ -16558,7 +16415,7 @@
     <row r="46" spans="2:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B46" s="35"/>
       <c r="C46" s="346" t="s">
-        <v>556</v>
+        <v>546</v>
       </c>
       <c r="E46" s="161"/>
       <c r="I46" s="21"/>
@@ -16566,14 +16423,14 @@
       <c r="L46" s="146"/>
       <c r="M46" s="294"/>
       <c r="O46" s="199" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="P46" s="221"/>
     </row>
     <row r="47" spans="2:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B47" s="35"/>
       <c r="C47" s="346" t="s">
-        <v>557</v>
+        <v>547</v>
       </c>
       <c r="E47" s="161"/>
       <c r="I47" s="21"/>
@@ -16581,14 +16438,14 @@
       <c r="L47" s="146"/>
       <c r="M47" s="54"/>
       <c r="O47" s="199" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="P47" s="221"/>
     </row>
     <row r="48" spans="2:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35"/>
       <c r="C48" s="346" t="s">
-        <v>558</v>
+        <v>548</v>
       </c>
       <c r="E48" s="161"/>
       <c r="I48" s="21"/>
@@ -16596,14 +16453,14 @@
       <c r="L48" s="147"/>
       <c r="M48" s="54"/>
       <c r="O48" s="199" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="P48" s="221"/>
     </row>
     <row r="49" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B49" s="35"/>
       <c r="C49" s="346" t="s">
-        <v>559</v>
+        <v>549</v>
       </c>
       <c r="E49" s="161"/>
       <c r="I49" s="21"/>
@@ -16611,7 +16468,7 @@
       <c r="L49" s="146"/>
       <c r="M49" s="54"/>
       <c r="O49" s="199" t="s">
-        <v>515</v>
+        <v>505</v>
       </c>
       <c r="P49" s="221"/>
       <c r="R49" s="292"/>
@@ -16619,7 +16476,7 @@
     <row r="50" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35"/>
       <c r="C50" s="346" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="E50" s="161"/>
       <c r="I50" s="21"/>
@@ -16627,7 +16484,7 @@
       <c r="L50" s="146"/>
       <c r="M50" s="54"/>
       <c r="O50" s="199" t="s">
-        <v>614</v>
+        <v>604</v>
       </c>
       <c r="P50" s="221"/>
       <c r="R50" s="292"/>
@@ -16675,7 +16532,7 @@
     <row r="53" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B53" s="35"/>
       <c r="C53" s="58" t="s">
-        <v>561</v>
+        <v>551</v>
       </c>
       <c r="D53" s="58"/>
       <c r="E53" s="61"/>
@@ -16688,7 +16545,7 @@
     <row r="54" spans="2:18" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B54" s="35"/>
       <c r="C54" s="346" t="s">
-        <v>556</v>
+        <v>546</v>
       </c>
       <c r="E54" s="181"/>
       <c r="I54" s="21"/>
@@ -16696,7 +16553,7 @@
       <c r="L54" s="146"/>
       <c r="M54" s="54"/>
       <c r="O54" s="199" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="P54" s="224"/>
       <c r="R54" s="292"/>
@@ -16704,7 +16561,7 @@
     <row r="55" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B55" s="35"/>
       <c r="C55" s="346" t="s">
-        <v>555</v>
+        <v>545</v>
       </c>
       <c r="E55" s="161"/>
       <c r="I55" s="21"/>
@@ -16712,7 +16569,7 @@
       <c r="L55" s="146"/>
       <c r="M55" s="54"/>
       <c r="O55" s="199" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="P55" s="224"/>
     </row>
@@ -16728,14 +16585,14 @@
       <c r="L56" s="146"/>
       <c r="M56" s="54"/>
       <c r="O56" s="199" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="P56" s="224"/>
     </row>
     <row r="57" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B57" s="35"/>
       <c r="C57" s="346" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="D57" s="58"/>
       <c r="E57" s="181"/>
@@ -16744,7 +16601,7 @@
       <c r="L57" s="146"/>
       <c r="M57" s="54"/>
       <c r="O57" s="199" t="s">
-        <v>615</v>
+        <v>605</v>
       </c>
       <c r="P57" s="224"/>
     </row>
@@ -16789,7 +16646,7 @@
     <row r="60" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B60" s="35"/>
       <c r="C60" s="1" t="s">
-        <v>562</v>
+        <v>552</v>
       </c>
       <c r="E60" s="57"/>
       <c r="K60" s="62"/>
@@ -16831,7 +16688,7 @@
     <row r="63" spans="2:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B63" s="35"/>
       <c r="C63" s="346" t="s">
-        <v>563</v>
+        <v>553</v>
       </c>
       <c r="E63" s="161"/>
       <c r="I63" s="21"/>
@@ -16861,7 +16718,7 @@
     </row>
     <row r="65" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B65" s="284" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="C65" s="51"/>
       <c r="D65" s="51"/>
@@ -16880,81 +16737,46 @@
     <row r="66" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B66" s="28"/>
       <c r="C66" s="1" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="E66" s="162">
         <v>1</v>
       </c>
       <c r="M66" s="29"/>
       <c r="O66" s="199" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="P66" s="7"/>
     </row>
     <row r="67" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B67" s="28"/>
       <c r="C67" s="1" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="E67" s="162">
         <v>0</v>
       </c>
       <c r="M67" s="29"/>
       <c r="O67" s="199" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="P67" s="7"/>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B68" s="28"/>
-      <c r="E68" s="162"/>
-      <c r="M68" s="29"/>
-      <c r="O68" s="199"/>
-      <c r="P68" s="7"/>
-    </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B69" s="28"/>
-      <c r="C69" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="E69" s="162">
-        <v>3.9E-2</v>
-      </c>
-      <c r="M69" s="29"/>
-      <c r="O69" s="199" t="s">
-        <v>510</v>
-      </c>
-      <c r="P69" s="7"/>
-    </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B70" s="28"/>
-      <c r="C70" s="1" t="s">
-        <v>492</v>
-      </c>
-      <c r="E70" s="162">
-        <v>5.2999999999999999E-2</v>
-      </c>
-      <c r="M70" s="29"/>
-      <c r="O70" s="199" t="s">
-        <v>511</v>
-      </c>
-      <c r="P70" s="7"/>
-    </row>
-    <row r="71" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="45"/>
-      <c r="C71" s="94"/>
-      <c r="D71" s="94"/>
-      <c r="E71" s="94"/>
-      <c r="F71" s="94"/>
-      <c r="G71" s="217"/>
-      <c r="H71" s="217"/>
-      <c r="I71" s="94"/>
-      <c r="J71" s="94"/>
-      <c r="K71" s="94"/>
-      <c r="L71" s="94"/>
-      <c r="M71" s="95"/>
-      <c r="O71" s="18"/>
-      <c r="P71" s="10"/>
+    <row r="68" spans="2:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="45"/>
+      <c r="C68" s="94"/>
+      <c r="D68" s="94"/>
+      <c r="E68" s="94"/>
+      <c r="F68" s="94"/>
+      <c r="G68" s="217"/>
+      <c r="H68" s="217"/>
+      <c r="I68" s="94"/>
+      <c r="J68" s="94"/>
+      <c r="K68" s="94"/>
+      <c r="L68" s="94"/>
+      <c r="M68" s="95"/>
+      <c r="O68" s="18"/>
+      <c r="P68" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -17100,7 +16922,7 @@
   <sheetData>
     <row r="2" spans="2:67" ht="21" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
     </row>
     <row r="3" spans="2:67" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23952,7 +23774,7 @@
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" s="375" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="C5" s="376"/>
       <c r="D5" s="376"/>
@@ -23967,15 +23789,15 @@
     <row r="6" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B7" s="303" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="C7" s="304"/>
       <c r="D7" s="304"/>
       <c r="E7" s="305" t="s">
-        <v>543</v>
+        <v>533</v>
       </c>
       <c r="F7" s="301" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="G7" s="300"/>
       <c r="H7" s="301"/>
@@ -23984,7 +23806,7 @@
       <c r="K7" s="51"/>
       <c r="L7" s="27"/>
       <c r="M7" s="243" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
     </row>
     <row r="8" spans="2:13" ht="34" x14ac:dyDescent="0.2">
@@ -23995,19 +23817,19 @@
         <v>225</v>
       </c>
       <c r="E8" s="318" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>522</v>
+        <v>512</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>523</v>
+        <v>513</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>523</v>
+        <v>513</v>
       </c>
       <c r="I8" s="309" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="J8" s="311" t="s">
         <v>228</v>
@@ -24025,16 +23847,16 @@
       <c r="D9" s="70"/>
       <c r="E9" s="310"/>
       <c r="F9" s="302" t="s">
-        <v>524</v>
+        <v>514</v>
       </c>
       <c r="G9" s="302" t="s">
-        <v>525</v>
+        <v>515</v>
       </c>
       <c r="H9" s="302" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>526</v>
+        <v>516</v>
       </c>
       <c r="J9" s="18"/>
       <c r="K9" s="9"/>
@@ -24062,17 +23884,17 @@
       </c>
       <c r="D11"/>
       <c r="E11" s="316" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="F11" s="326"/>
       <c r="G11" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H11" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I11" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J11" s="335">
         <f>F11</f>
@@ -24084,7 +23906,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="243" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
@@ -24094,15 +23916,15 @@
       </c>
       <c r="D12"/>
       <c r="E12" s="316" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="F12" s="326"/>
       <c r="G12" s="326"/>
       <c r="H12" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I12" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J12" s="335"/>
       <c r="K12" s="321" t="e">
@@ -24114,7 +23936,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M12" s="243" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
@@ -24124,15 +23946,15 @@
       </c>
       <c r="D13"/>
       <c r="E13" s="316" t="s">
-        <v>529</v>
+        <v>519</v>
       </c>
       <c r="F13" s="326"/>
       <c r="G13" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H13" s="326"/>
       <c r="I13" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J13" s="335"/>
       <c r="K13" s="321" t="e">
@@ -24144,7 +23966,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M13" s="243" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.2">
@@ -24154,17 +23976,17 @@
       </c>
       <c r="D14"/>
       <c r="E14" s="316" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="F14" s="326"/>
       <c r="G14" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H14" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I14" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J14" s="335">
         <f>F14</f>
@@ -24176,7 +23998,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="243" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
@@ -24186,17 +24008,17 @@
       </c>
       <c r="D15"/>
       <c r="E15" s="316" t="s">
-        <v>531</v>
+        <v>521</v>
       </c>
       <c r="F15" s="326"/>
       <c r="G15" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H15" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I15" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J15" s="335">
         <f>F15</f>
@@ -24208,7 +24030,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="243" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.2">
@@ -24218,17 +24040,17 @@
       </c>
       <c r="D16"/>
       <c r="E16" s="316" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
       <c r="F16" s="326"/>
       <c r="G16" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H16" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I16" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J16" s="335">
         <f>F16</f>
@@ -24240,25 +24062,25 @@
         <v>0</v>
       </c>
       <c r="M16" s="243" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" s="69"/>
       <c r="C17" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="D17"/>
       <c r="E17" s="316" t="s">
-        <v>611</v>
+        <v>601</v>
       </c>
       <c r="F17" s="326"/>
       <c r="G17" s="326"/>
       <c r="H17" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I17" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J17" s="335"/>
       <c r="K17" s="321" t="e">
@@ -24270,7 +24092,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M17" s="243" t="s">
-        <v>613</v>
+        <v>603</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
@@ -24292,17 +24114,17 @@
       </c>
       <c r="D19"/>
       <c r="E19" s="316" t="s">
-        <v>616</v>
+        <v>606</v>
       </c>
       <c r="F19" s="326"/>
       <c r="G19" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H19" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I19" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J19" s="335">
         <f>F19</f>
@@ -24314,7 +24136,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="243" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
@@ -24324,17 +24146,17 @@
       </c>
       <c r="D20"/>
       <c r="E20" s="316" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="F20" s="326"/>
       <c r="G20" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H20" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I20" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J20" s="335">
         <f>F20</f>
@@ -24346,7 +24168,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="243" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
@@ -24356,17 +24178,17 @@
       </c>
       <c r="D21"/>
       <c r="E21" s="316" t="s">
-        <v>618</v>
+        <v>608</v>
       </c>
       <c r="F21" s="326"/>
       <c r="G21" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H21" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I21" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J21" s="335">
         <f>F21</f>
@@ -24378,7 +24200,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="243" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.2">
@@ -24415,17 +24237,17 @@
       </c>
       <c r="D24"/>
       <c r="E24" s="316" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
       <c r="F24" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G24" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H24" s="326"/>
       <c r="I24" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J24" s="335"/>
       <c r="K24" s="321" t="e">
@@ -24437,7 +24259,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M24" s="243" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.2">
@@ -24447,17 +24269,17 @@
       </c>
       <c r="D25"/>
       <c r="E25" s="316" t="s">
-        <v>535</v>
+        <v>525</v>
       </c>
       <c r="F25" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G25" s="326"/>
       <c r="H25" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I25" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J25" s="335"/>
       <c r="K25" s="321" t="e">
@@ -24469,7 +24291,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M25" s="243" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.2">
@@ -24479,17 +24301,17 @@
       </c>
       <c r="D26"/>
       <c r="E26" s="316" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="F26" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G26" s="326"/>
       <c r="H26" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I26" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J26" s="335"/>
       <c r="K26" s="321" t="e">
@@ -24501,27 +24323,27 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M26" s="243" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B27" s="69"/>
       <c r="C27" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="D27"/>
       <c r="E27" s="316" t="s">
-        <v>609</v>
+        <v>599</v>
       </c>
       <c r="F27" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G27" s="326"/>
       <c r="H27" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I27" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="J27" s="335"/>
       <c r="K27" s="321" t="e">
@@ -24533,7 +24355,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="M27" s="243" t="s">
-        <v>610</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.2">
@@ -24569,16 +24391,16 @@
       </c>
       <c r="D30"/>
       <c r="E30" s="316" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="F30" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G30" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H30" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I30" s="326"/>
       <c r="J30" s="335">
@@ -24591,7 +24413,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="243" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.2">
@@ -24601,16 +24423,16 @@
       </c>
       <c r="D31"/>
       <c r="E31" s="316" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="F31" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="G31" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H31" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I31" s="326"/>
       <c r="J31" s="335">
@@ -24623,7 +24445,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="243" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.2">
@@ -24633,16 +24455,16 @@
       </c>
       <c r="D32"/>
       <c r="E32" s="316" t="s">
+        <v>529</v>
+      </c>
+      <c r="F32" s="326" t="s">
         <v>539</v>
       </c>
-      <c r="F32" s="326" t="s">
-        <v>549</v>
-      </c>
       <c r="G32" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="H32" s="326" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
       <c r="I32" s="326"/>
       <c r="J32" s="335">
@@ -24655,7 +24477,7 @@
         <v>0</v>
       </c>
       <c r="M32" s="243" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="33" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>